<commit_message>
test: add historical Resource Viewer coverage
</commit_message>
<xml_diff>
--- a/docs/tcm-import-resource-viewer.xlsx
+++ b/docs/tcm-import-resource-viewer.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Meta" sheetId="1" r:id="R0e347c303cc944b7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Features" sheetId="2" r:id="Raf484fb7aa6d46e7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AcceptanceCriteria" sheetId="3" r:id="Rf2e002184d6e4ea0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TestCases" sheetId="4" r:id="R76210caebbd544ed"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Steps" sheetId="5" r:id="R585de4d9a5fb42a9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DatasetSchema" sheetId="6" r:id="Rd04438c7957e484b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ParameterSets" sheetId="7" r:id="Rd916527d4eeb4157"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AutomationLinks" sheetId="8" r:id="Rfe96e32f59aa448c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CrossFeatures" sheetId="9" r:id="Rbc955ab90e23417e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Meta" sheetId="1" r:id="R90689e4a57e745c6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Features" sheetId="2" r:id="R0fd3e77a9bd44388"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AcceptanceCriteria" sheetId="3" r:id="Rddd026c1545b4c29"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TestCases" sheetId="4" r:id="Rf48fda9a7aef4527"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Steps" sheetId="5" r:id="R18f4f5c6acb2421f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DatasetSchema" sheetId="6" r:id="Rbcc81bf355d5437d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ParameterSets" sheetId="7" r:id="R7eac9eace6e84091"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AutomationLinks" sheetId="8" r:id="R0d562c6624ba4304"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CrossFeatures" sheetId="9" r:id="Rae26af7b66d5422d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1051,6 +1051,20 @@
         <x:v>2</x:v>
       </x:c>
     </x:row>
+    <x:row r="31">
+      <x:c r="A31" t="str">
+        <x:v>REQ-RVW-BOM</x:v>
+      </x:c>
+      <x:c r="B31" t="str">
+        <x:v>AC-15</x:v>
+      </x:c>
+      <x:c r="C31" t="str">
+        <x:v>Якщо на момент переміщення не існувало жодної tech map, ресурс залишається атомарним; карта, створена пізніше, на нього не впливає.</x:v>
+      </x:c>
+      <x:c r="D31" t="str">
+        <x:v>14</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -2813,6 +2827,104 @@
       </x:c>
       <x:c r="Q35" t="str"/>
     </x:row>
+    <x:row r="36">
+      <x:c r="A36" t="str">
+        <x:v>TC-RVW-BOM-035</x:v>
+      </x:c>
+      <x:c r="B36" t="str">
+        <x:v>REQ-RVW-BOM</x:v>
+      </x:c>
+      <x:c r="C36" t="str">
+        <x:v>AC-15</x:v>
+      </x:c>
+      <x:c r="D36" t="str">
+        <x:v>BOM — до першої tech map ресурс атомарний</x:v>
+      </x:c>
+      <x:c r="E36" t="str">
+        <x:v>Мета: Якщо на момент переміщення не існувало жодної tech map, пізніше створена карта не змінює історичний склад.</x:v>
+      </x:c>
+      <x:c r="F36" t="str">
+        <x:v>HIGH</x:v>
+      </x:c>
+      <x:c r="G36" t="str">
+        <x:v>CRITICAL</x:v>
+      </x:c>
+      <x:c r="H36" t="str">
+        <x:v>ACTIVE</x:v>
+      </x:c>
+      <x:c r="I36" t="str">
+        <x:v>FUNCTIONAL</x:v>
+      </x:c>
+      <x:c r="J36" t="str">
+        <x:v>@ResourceViewer (wolf) залогінений. Середовище dev/staging. @Admin підготував техкарти PRODUCTION + stock на OWNER_1 storage; receiver = UNIT storage.</x:v>
+      </x:c>
+      <x:c r="K36" t="str">
+        <x:v>Component відсутній; Product лишається атомарним, isProduct=false</x:v>
+      </x:c>
+      <x:c r="L36" t="str">
+        <x:v>resource-viewer,api</x:v>
+      </x:c>
+      <x:c r="M36" t="str">
+        <x:v>QA</x:v>
+      </x:c>
+      <x:c r="N36"/>
+      <x:c r="O36" t="str">
+        <x:v>ResourceViewer</x:v>
+      </x:c>
+      <x:c r="P36" t="str">
+        <x:v>false</x:v>
+      </x:c>
+      <x:c r="Q36"/>
+    </x:row>
+    <x:row r="37">
+      <x:c r="A37" t="str">
+        <x:v>TC-RVW-BOM-036</x:v>
+      </x:c>
+      <x:c r="B37" t="str">
+        <x:v>REQ-RVW-BOM</x:v>
+      </x:c>
+      <x:c r="C37" t="str">
+        <x:v>AC-15</x:v>
+      </x:c>
+      <x:c r="D37" t="str">
+        <x:v>BOM — зовнішня партія до першої tech map атомарна</x:v>
+      </x:c>
+      <x:c r="E37" t="str">
+        <x:v>Мета: Зовнішньо отримана партія, переміщена до появи першої tech map, лишається атомарною; пізніше створена карта не змінює історичний склад.</x:v>
+      </x:c>
+      <x:c r="F37" t="str">
+        <x:v>HIGH</x:v>
+      </x:c>
+      <x:c r="G37" t="str">
+        <x:v>CRITICAL</x:v>
+      </x:c>
+      <x:c r="H37" t="str">
+        <x:v>ACTIVE</x:v>
+      </x:c>
+      <x:c r="I37" t="str">
+        <x:v>FUNCTIONAL</x:v>
+      </x:c>
+      <x:c r="J37" t="str">
+        <x:v>@ResourceViewer (wolf) залогінений. Середовище dev/staging. @Admin підготував техкарти PRODUCTION + stock на OWNER_1 storage; receiver = UNIT storage.</x:v>
+      </x:c>
+      <x:c r="K37" t="str">
+        <x:v>Один атомарний рядок Product, isProduct=false</x:v>
+      </x:c>
+      <x:c r="L37" t="str">
+        <x:v>resource-viewer,api</x:v>
+      </x:c>
+      <x:c r="M37" t="str">
+        <x:v>QA</x:v>
+      </x:c>
+      <x:c r="N37"/>
+      <x:c r="O37" t="str">
+        <x:v>ResourceViewer</x:v>
+      </x:c>
+      <x:c r="P37" t="str">
+        <x:v>false</x:v>
+      </x:c>
+      <x:c r="Q37"/>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -3824,6 +3936,104 @@
         <x:v>є product і ingredient рядки для Alcohol</x:v>
       </x:c>
     </x:row>
+    <x:row r="72">
+      <x:c r="A72" t="str">
+        <x:v>TC-RVW-BOM-035</x:v>
+      </x:c>
+      <x:c r="B72" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C72" t="str">
+        <x:v>Створити inventory stock Product і перемістити його до появи tech map</x:v>
+      </x:c>
+      <x:c r="D72" t="str">
+        <x:v>relocationId</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="73">
+      <x:c r="A73" t="str">
+        <x:v>TC-RVW-BOM-035</x:v>
+      </x:c>
+      <x:c r="B73" t="str">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C73" t="str">
+        <x:v>Після переміщення створити tech map Product←Component</x:v>
+      </x:c>
+      <x:c r="D73" t="str">
+        <x:v>Tech map створена пізніше</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="74">
+      <x:c r="A74" t="str">
+        <x:v>TC-RVW-BOM-035</x:v>
+      </x:c>
+      <x:c r="B74" t="str">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C74" t="str">
+        <x:v>GET journal/sum</x:v>
+      </x:c>
+      <x:c r="D74" t="str">
+        <x:v>Component відсутній; Product лишається атомарним, isProduct=false</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="75">
+      <x:c r="A75" t="str">
+        <x:v>TC-RVW-BOM-036</x:v>
+      </x:c>
+      <x:c r="B75" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C75" t="str">
+        <x:v>Отримати Product зовнішньою партією та перемістити її до появи tech map</x:v>
+      </x:c>
+      <x:c r="D75" t="str">
+        <x:v>relocationId; isProduced=false</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="76">
+      <x:c r="A76" t="str">
+        <x:v>TC-RVW-BOM-036</x:v>
+      </x:c>
+      <x:c r="B76" t="str">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C76" t="str">
+        <x:v>Після переміщення створити tech map Product←Component</x:v>
+      </x:c>
+      <x:c r="D76" t="str">
+        <x:v>Tech map створена пізніше</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="77">
+      <x:c r="A77" t="str">
+        <x:v>TC-RVW-BOM-036</x:v>
+      </x:c>
+      <x:c r="B77" t="str">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C77" t="str">
+        <x:v>GET journal/sum за Component</x:v>
+      </x:c>
+      <x:c r="D77" t="str">
+        <x:v>Relocation відсутній; Component amount=0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="78">
+      <x:c r="A78" t="str">
+        <x:v>TC-RVW-BOM-036</x:v>
+      </x:c>
+      <x:c r="B78" t="str">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C78" t="str">
+        <x:v>GET journal за Product</x:v>
+      </x:c>
+      <x:c r="D78" t="str">
+        <x:v>Один атомарний рядок Product, isProduct=false</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -4403,6 +4613,34 @@
         <x:v>0</x:v>
       </x:c>
     </x:row>
+    <x:row r="36">
+      <x:c r="A36" t="str">
+        <x:v>TC-RVW-BOM-035</x:v>
+      </x:c>
+      <x:c r="B36" t="str">
+        <x:v>API</x:v>
+      </x:c>
+      <x:c r="C36" t="str">
+        <x:v>TC-RVW-BOM-035</x:v>
+      </x:c>
+      <x:c r="D36" t="str">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37">
+      <x:c r="A37" t="str">
+        <x:v>TC-RVW-BOM-036</x:v>
+      </x:c>
+      <x:c r="B37" t="str">
+        <x:v>API</x:v>
+      </x:c>
+      <x:c r="C37" t="str">
+        <x:v>TC-RVW-BOM-036</x:v>
+      </x:c>
+      <x:c r="D37" t="str">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -4696,6 +4934,22 @@
         <x:v>resource-viewer</x:v>
       </x:c>
     </x:row>
+    <x:row r="36">
+      <x:c r="A36" t="str">
+        <x:v>TC-RVW-BOM-035</x:v>
+      </x:c>
+      <x:c r="B36" t="str">
+        <x:v>resource-viewer</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37">
+      <x:c r="A37" t="str">
+        <x:v>TC-RVW-BOM-036</x:v>
+      </x:c>
+      <x:c r="B37" t="str">
+        <x:v>resource-viewer</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>